<commit_message>
quicksave before trying something
</commit_message>
<xml_diff>
--- a/onsets_edit.xlsx
+++ b/onsets_edit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brandonwoosnyder/Dropbox/docs-d/00_UCI_2025-2026/02_UCI_Winter_2026/Independent Study Rajna - Music 299/Constrained_PhoneGuide_Score/ScreenTimeScore/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{305A3D76-5BEF-CE42-A467-C8D6CDCBFAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CADD9A4-F67A-8A4F-8662-F187C0B00684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="180" yWindow="840" windowWidth="30060" windowHeight="17180" xr2:uid="{656903FE-55D6-334E-8317-D02588440573}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="68">
   <si>
     <t>onset_ms_1</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>IS THIS VALUE BELOW CORRECT???</t>
+  </si>
+  <si>
+    <t>bacon01bright</t>
   </si>
 </sst>
 </file>
@@ -1094,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E707C8EF-5282-2B42-BB2D-C2C257FF5AA3}">
-  <dimension ref="A1:S84"/>
+  <dimension ref="A1:S85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
@@ -1677,1030 +1680,1029 @@
         <v>64</v>
       </c>
       <c r="P12">
+        <f>P2+1</f>
         <v>2</v>
       </c>
       <c r="Q12">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13">
         <f>A12+($Q12*1000)</f>
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D13">
         <f>D12+($Q12*1000)</f>
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="E13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G13">
         <f>G12+($Q12*1000)</f>
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="H13" t="s">
-        <v>19</v>
-      </c>
-      <c r="I13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J13">
         <f>J12+($Q12*1000)</f>
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="K13" t="s">
-        <v>19</v>
-      </c>
-      <c r="L13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="M13">
         <f>M12+($Q12*1000)</f>
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="N13" t="s">
-        <v>19</v>
-      </c>
-      <c r="O13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="P13">
+        <f>P12+1</f>
         <v>3</v>
       </c>
       <c r="Q13">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14">
         <f>A13+($Q13*1000)</f>
-        <v>76000</v>
+        <v>50000</v>
       </c>
       <c r="B14" t="s">
         <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="D14">
         <f>D13+($Q13*1000)</f>
-        <v>76000</v>
+        <v>50000</v>
       </c>
       <c r="E14" t="s">
         <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="G14">
         <f>G13+($Q13*1000)</f>
-        <v>76000</v>
+        <v>50000</v>
       </c>
       <c r="H14" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I14" t="s">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="J14">
         <f>J13+($Q13*1000)</f>
-        <v>76000</v>
+        <v>50000</v>
       </c>
       <c r="K14" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L14" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="M14">
         <f>M13+($Q13*1000)</f>
-        <v>76000</v>
+        <v>50000</v>
       </c>
       <c r="N14" t="s">
         <v>19</v>
       </c>
       <c r="O14" t="s">
+        <v>65</v>
+      </c>
+      <c r="P14">
+        <f>P13+1</f>
+        <v>4</v>
+      </c>
+      <c r="Q14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <f>A14+($Q14*1000)</f>
+        <v>56000</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
         <v>30</v>
       </c>
-      <c r="P14">
-        <v>4</v>
-      </c>
-      <c r="Q14">
+      <c r="D15">
+        <f>D14+($Q14*1000)</f>
+        <v>56000</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15">
+        <f>G14+($Q14*1000)</f>
+        <v>56000</v>
+      </c>
+      <c r="H15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" t="s">
+        <v>32</v>
+      </c>
+      <c r="J15">
+        <f>J14+($Q14*1000)</f>
+        <v>56000</v>
+      </c>
+      <c r="K15" t="s">
+        <v>31</v>
+      </c>
+      <c r="L15" t="s">
+        <v>33</v>
+      </c>
+      <c r="M15">
+        <f>M14+($Q14*1000)</f>
+        <v>56000</v>
+      </c>
+      <c r="N15" t="s">
+        <v>19</v>
+      </c>
+      <c r="O15" t="s">
+        <v>30</v>
+      </c>
+      <c r="P15">
+        <f>P14+1</f>
+        <v>5</v>
+      </c>
+      <c r="Q15">
         <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="G15">
-        <f t="shared" ref="G15:G20" si="0">G14+($S$2)</f>
-        <v>80000</v>
-      </c>
-      <c r="H15" t="s">
-        <v>19</v>
-      </c>
-      <c r="I15" t="s">
-        <v>34</v>
-      </c>
-      <c r="J15">
-        <f t="shared" ref="J15:J26" si="1">J14+($S$2*(1+$R$2))</f>
-        <v>80050</v>
-      </c>
-      <c r="K15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L15" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G16">
-        <f t="shared" si="0"/>
-        <v>84000</v>
+        <f t="shared" ref="G16:G21" si="0">G15+($S$2)</f>
+        <v>60000</v>
       </c>
       <c r="H16" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J16">
-        <f t="shared" si="1"/>
-        <v>84100</v>
+        <f t="shared" ref="J16:J27" si="1">J15+($S$2*(1+$R$2))</f>
+        <v>60050</v>
       </c>
       <c r="K16" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L16" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G17">
         <f t="shared" si="0"/>
-        <v>88000</v>
+        <v>64000</v>
       </c>
       <c r="H17" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I17" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J17">
         <f t="shared" si="1"/>
-        <v>88150</v>
+        <v>64100</v>
       </c>
       <c r="K17" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G18">
         <f t="shared" si="0"/>
-        <v>92000</v>
+        <v>68000</v>
       </c>
       <c r="H18" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J18">
         <f t="shared" si="1"/>
-        <v>92200</v>
+        <v>68150</v>
       </c>
       <c r="K18" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L18" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G19">
         <f t="shared" si="0"/>
-        <v>96000</v>
+        <v>72000</v>
       </c>
       <c r="H19" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I19" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J19">
         <f t="shared" si="1"/>
-        <v>96250</v>
+        <v>72200</v>
       </c>
       <c r="K19" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A20">
-        <f>A14+($Q14*1000)</f>
-        <v>100000</v>
-      </c>
-      <c r="B20" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20">
-        <f>D14+($Q14*1000)</f>
-        <v>100000</v>
-      </c>
-      <c r="E20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F20" t="s">
-        <v>36</v>
-      </c>
       <c r="G20">
         <f t="shared" si="0"/>
-        <v>100000</v>
+        <v>76000</v>
       </c>
       <c r="H20" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J20">
         <f t="shared" si="1"/>
-        <v>100300</v>
+        <v>76250</v>
       </c>
       <c r="K20" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M20">
-        <f>M14+($Q14*1000)</f>
-        <v>100000</v>
-      </c>
-      <c r="N20" t="s">
-        <v>19</v>
-      </c>
-      <c r="O20" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <f>A15+($Q15*1000)</f>
+        <v>80000</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" t="s">
         <v>36</v>
       </c>
-      <c r="P20">
-        <v>5</v>
-      </c>
-      <c r="Q20">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="D21">
+        <f>D15+($Q15*1000)</f>
+        <v>80000</v>
+      </c>
+      <c r="E21" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" t="s">
+        <v>36</v>
+      </c>
       <c r="G21">
-        <f t="shared" ref="G21:G39" si="2">G20+($S$2)</f>
-        <v>104000</v>
+        <f t="shared" si="0"/>
+        <v>80000</v>
       </c>
       <c r="H21" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J21">
         <f t="shared" si="1"/>
-        <v>104350</v>
+        <v>80300</v>
       </c>
       <c r="K21" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L21" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="M21">
+        <f>M15+($Q15*1000)</f>
+        <v>80000</v>
+      </c>
+      <c r="N21" t="s">
+        <v>19</v>
+      </c>
+      <c r="O21" t="s">
+        <v>36</v>
+      </c>
+      <c r="P21">
+        <f>P15+1</f>
+        <v>6</v>
+      </c>
+      <c r="Q21">
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G22">
-        <f t="shared" si="2"/>
-        <v>108000</v>
+        <f t="shared" ref="G22:G40" si="2">G21+($S$2)</f>
+        <v>84000</v>
       </c>
       <c r="H22" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I22" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J22">
         <f t="shared" si="1"/>
-        <v>108400</v>
+        <v>84350</v>
       </c>
       <c r="K22" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L22" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G23">
         <f t="shared" si="2"/>
-        <v>112000</v>
+        <v>88000</v>
       </c>
       <c r="H23" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J23">
         <f t="shared" si="1"/>
-        <v>112450</v>
+        <v>88400</v>
       </c>
       <c r="K23" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G24">
         <f t="shared" si="2"/>
-        <v>116000</v>
+        <v>92000</v>
       </c>
       <c r="H24" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I24" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J24">
         <f t="shared" si="1"/>
-        <v>116500</v>
+        <v>92450</v>
       </c>
       <c r="K24" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L24" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G25">
         <f t="shared" si="2"/>
-        <v>120000</v>
+        <v>96000</v>
       </c>
       <c r="H25" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J25">
         <f t="shared" si="1"/>
-        <v>120550</v>
+        <v>96500</v>
       </c>
       <c r="K25" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L25" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G26">
         <f t="shared" si="2"/>
-        <v>124000</v>
+        <v>100000</v>
       </c>
       <c r="H26" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I26" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J26">
         <f t="shared" si="1"/>
-        <v>124600</v>
+        <v>100550</v>
       </c>
       <c r="K26" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L26" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <f>A20+($Q20*1000)</f>
-        <v>128000</v>
-      </c>
-      <c r="B27" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" t="s">
-        <v>36</v>
-      </c>
-      <c r="D27">
-        <f>D20+($Q20*1000)</f>
-        <v>128000</v>
-      </c>
-      <c r="E27" t="s">
-        <v>19</v>
-      </c>
-      <c r="F27" t="s">
-        <v>36</v>
-      </c>
       <c r="G27">
         <f t="shared" si="2"/>
-        <v>128000</v>
+        <v>104000</v>
       </c>
       <c r="H27" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I27" t="s">
-        <v>34</v>
-      </c>
-      <c r="M27">
-        <f>M20+($Q20*1000)</f>
-        <v>128000</v>
-      </c>
-      <c r="N27" t="s">
-        <v>19</v>
-      </c>
-      <c r="O27" t="s">
+        <v>32</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="1"/>
+        <v>104600</v>
+      </c>
+      <c r="K27" t="s">
+        <v>31</v>
+      </c>
+      <c r="L27" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <f>A21+($Q21*1000)</f>
+        <v>108000</v>
+      </c>
+      <c r="B28" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" t="s">
         <v>36</v>
       </c>
-      <c r="P27">
-        <v>6</v>
-      </c>
-      <c r="Q27">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="D28">
+        <f>D21+($Q21*1000)</f>
+        <v>108000</v>
+      </c>
+      <c r="E28" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" t="s">
+        <v>36</v>
+      </c>
       <c r="G28">
         <f t="shared" si="2"/>
-        <v>132000</v>
+        <v>108000</v>
       </c>
       <c r="H28" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I28" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+      <c r="M28">
+        <f>M21+($Q21*1000)</f>
+        <v>108000</v>
+      </c>
+      <c r="N28" t="s">
+        <v>19</v>
+      </c>
+      <c r="O28" t="s">
+        <v>36</v>
+      </c>
+      <c r="P28">
+        <f>P21+1</f>
+        <v>7</v>
+      </c>
+      <c r="Q28">
+        <v>28</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G29">
         <f t="shared" si="2"/>
-        <v>136000</v>
+        <v>112000</v>
       </c>
       <c r="H29" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I29" t="s">
-        <v>34</v>
-      </c>
-      <c r="J29">
-        <f>J26+(11000)</f>
-        <v>135600</v>
-      </c>
-      <c r="K29" t="s">
-        <v>19</v>
-      </c>
-      <c r="L29" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G30">
         <f t="shared" si="2"/>
-        <v>140000</v>
+        <v>116000</v>
       </c>
       <c r="H30" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I30" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J30">
-        <f>J29+2000</f>
-        <v>137600</v>
+        <f>J27+(11000)</f>
+        <v>115600</v>
       </c>
       <c r="K30" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G31">
         <f t="shared" si="2"/>
-        <v>144000</v>
+        <v>120000</v>
       </c>
       <c r="H31" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J31">
-        <f>J30+4000</f>
-        <v>141600</v>
+        <f>J30+2000</f>
+        <v>117600</v>
       </c>
       <c r="K31" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L31" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="G32">
         <f t="shared" si="2"/>
-        <v>148000</v>
+        <v>124000</v>
       </c>
       <c r="H32" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I32" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+      <c r="J32">
+        <f>J31+4000</f>
+        <v>121600</v>
+      </c>
+      <c r="K32" t="s">
+        <v>19</v>
+      </c>
+      <c r="L32" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="G33">
         <f t="shared" si="2"/>
-        <v>152000</v>
+        <v>128000</v>
       </c>
       <c r="H33" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I33" t="s">
-        <v>34</v>
-      </c>
-      <c r="J33">
-        <f>J31+11000</f>
-        <v>152600</v>
-      </c>
-      <c r="K33" t="s">
-        <v>19</v>
-      </c>
-      <c r="L33" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34">
-        <f>A27+($Q27*1000)</f>
-        <v>156000</v>
-      </c>
-      <c r="B34" t="s">
-        <v>19</v>
-      </c>
-      <c r="C34" t="s">
-        <v>40</v>
-      </c>
-      <c r="D34">
-        <f>D27+($Q27*1000)</f>
-        <v>156000</v>
-      </c>
-      <c r="E34" t="s">
-        <v>19</v>
-      </c>
-      <c r="F34" t="s">
-        <v>40</v>
-      </c>
       <c r="G34">
         <f t="shared" si="2"/>
-        <v>156000</v>
+        <v>132000</v>
       </c>
       <c r="H34" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I34" t="s">
-        <v>32</v>
-      </c>
-      <c r="M34">
-        <f>M27+($Q27*1000)</f>
-        <v>156000</v>
-      </c>
-      <c r="N34" t="s">
-        <v>19</v>
-      </c>
-      <c r="O34" t="s">
+        <v>34</v>
+      </c>
+      <c r="J34">
+        <f>J32+11000</f>
+        <v>132600</v>
+      </c>
+      <c r="K34" t="s">
+        <v>19</v>
+      </c>
+      <c r="L34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <f>A28+($Q28*1000)</f>
+        <v>136000</v>
+      </c>
+      <c r="B35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" t="s">
         <v>40</v>
       </c>
-      <c r="P34">
-        <v>7</v>
-      </c>
-      <c r="Q34">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <f>D28+($Q28*1000)</f>
+        <v>136000</v>
+      </c>
+      <c r="E35" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" t="s">
+        <v>40</v>
+      </c>
       <c r="G35">
         <f t="shared" si="2"/>
-        <v>160000</v>
+        <v>136000</v>
       </c>
       <c r="H35" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I35" t="s">
-        <v>34</v>
-      </c>
-      <c r="J35">
-        <f>G35</f>
-        <v>160000</v>
-      </c>
-      <c r="K35" t="s">
-        <v>31</v>
-      </c>
-      <c r="L35" t="s">
         <v>32</v>
+      </c>
+      <c r="M35">
+        <f>M28+($Q28*1000)</f>
+        <v>136000</v>
+      </c>
+      <c r="N35" t="s">
+        <v>19</v>
+      </c>
+      <c r="O35" t="s">
+        <v>40</v>
+      </c>
+      <c r="P35">
+        <f>P28+1</f>
+        <v>8</v>
+      </c>
+      <c r="Q35">
+        <v>12</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.2">
       <c r="G36">
-        <f>G35+($S$2)</f>
-        <v>164000</v>
+        <f t="shared" si="2"/>
+        <v>140000</v>
       </c>
       <c r="H36" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I36" t="s">
+        <v>34</v>
+      </c>
+      <c r="J36">
+        <f>G36</f>
+        <v>140000</v>
+      </c>
+      <c r="K36" t="s">
+        <v>31</v>
+      </c>
+      <c r="L36" t="s">
         <v>32</v>
-      </c>
-      <c r="J36">
-        <f>J35+($S$2)</f>
-        <v>164000</v>
-      </c>
-      <c r="K36" t="s">
-        <v>19</v>
-      </c>
-      <c r="L36" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.2">
       <c r="G37">
         <f>G36+($S$2)</f>
-        <v>168000</v>
+        <v>144000</v>
       </c>
       <c r="H37" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I37" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J37">
         <f>J36+($S$2)</f>
-        <v>168000</v>
+        <v>144000</v>
       </c>
       <c r="K37" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L37" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="G38">
-        <f t="shared" si="2"/>
-        <v>172000</v>
+        <f>G37+($S$2)</f>
+        <v>148000</v>
       </c>
       <c r="H38" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I38" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J38">
         <f>J37+($S$2)</f>
-        <v>172000</v>
+        <v>148000</v>
       </c>
       <c r="K38" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A39">
-        <f>A34+($Q34*1000)</f>
-        <v>168000</v>
-      </c>
-      <c r="B39" t="s">
-        <v>19</v>
-      </c>
-      <c r="C39" t="s">
-        <v>41</v>
-      </c>
-      <c r="D39">
-        <f>D34+($Q34*1000)</f>
-        <v>168000</v>
-      </c>
-      <c r="E39" t="s">
-        <v>19</v>
-      </c>
-      <c r="F39" t="s">
-        <v>41</v>
-      </c>
       <c r="G39">
         <f t="shared" si="2"/>
-        <v>176000</v>
+        <v>152000</v>
       </c>
       <c r="H39" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I39" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="J39">
         <f>J38+($S$2)</f>
-        <v>176000</v>
+        <v>152000</v>
       </c>
       <c r="K39" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L39" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <f>A35+($Q35*1000)</f>
+        <v>148000</v>
+      </c>
+      <c r="B40" t="s">
+        <v>19</v>
+      </c>
+      <c r="C40" t="s">
+        <v>41</v>
+      </c>
+      <c r="D40">
+        <f>D35+($Q35*1000)</f>
+        <v>148000</v>
+      </c>
+      <c r="E40" t="s">
+        <v>19</v>
+      </c>
+      <c r="F40" t="s">
+        <v>41</v>
+      </c>
+      <c r="G40">
+        <f t="shared" si="2"/>
+        <v>156000</v>
+      </c>
+      <c r="H40" t="s">
+        <v>19</v>
+      </c>
+      <c r="I40" t="s">
+        <v>42</v>
+      </c>
+      <c r="J40">
+        <f>J39+($S$2)</f>
+        <v>156000</v>
+      </c>
+      <c r="K40" t="s">
+        <v>31</v>
+      </c>
+      <c r="L40" t="s">
         <v>39</v>
       </c>
-      <c r="M39">
-        <f>M34+($Q34*1000)</f>
-        <v>168000</v>
-      </c>
-      <c r="N39" t="s">
-        <v>19</v>
-      </c>
-      <c r="O39" t="s">
+      <c r="M40">
+        <f>M35+($Q35*1000)</f>
+        <v>148000</v>
+      </c>
+      <c r="N40" t="s">
+        <v>19</v>
+      </c>
+      <c r="O40" t="s">
         <v>41</v>
       </c>
-      <c r="P39">
-        <v>8</v>
-      </c>
-      <c r="Q39">
+      <c r="P40">
+        <f>P35+1</f>
+        <v>9</v>
+      </c>
+      <c r="Q40">
         <v>10</v>
-      </c>
-    </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="J40">
-        <f>J39+1000</f>
-        <v>177000</v>
-      </c>
-      <c r="K40" t="s">
-        <v>19</v>
-      </c>
-      <c r="L40" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J41">
-        <f>J40+3000</f>
-        <v>180000</v>
+        <f>J40+1000</f>
+        <v>157000</v>
       </c>
       <c r="K41" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L41" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="J42">
+        <f>J41+3000</f>
+        <v>160000</v>
+      </c>
+      <c r="K42" t="s">
+        <v>31</v>
+      </c>
+      <c r="L42" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A42">
-        <f>A39+($Q39*1000)</f>
-        <v>178000</v>
-      </c>
-      <c r="B42" t="s">
-        <v>19</v>
-      </c>
-      <c r="C42" t="s">
-        <v>44</v>
-      </c>
-      <c r="D42">
-        <f>D39+($Q39*1000)</f>
-        <v>178000</v>
-      </c>
-      <c r="E42" t="s">
-        <v>19</v>
-      </c>
-      <c r="F42" t="s">
-        <v>65</v>
-      </c>
-      <c r="G42">
-        <f>G39+Q39*1000</f>
-        <v>186000</v>
-      </c>
-      <c r="H42" t="s">
-        <v>31</v>
-      </c>
-      <c r="I42" t="s">
-        <v>43</v>
-      </c>
-      <c r="J42">
-        <f>J41+6000</f>
-        <v>186000</v>
-      </c>
-      <c r="K42" t="s">
-        <v>19</v>
-      </c>
-      <c r="L42" t="s">
-        <v>43</v>
-      </c>
-      <c r="M42">
-        <f>M39+($Q39*1000)</f>
-        <v>178000</v>
-      </c>
-      <c r="N42" t="s">
-        <v>19</v>
-      </c>
-      <c r="O42" t="s">
-        <v>65</v>
-      </c>
-      <c r="P42">
-        <v>9</v>
-      </c>
-      <c r="Q42">
-        <v>6</v>
-      </c>
-      <c r="R42" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A43">
-        <f t="shared" ref="A43:A48" si="3">A42+($Q42*1000)</f>
-        <v>184000</v>
+        <f>A40+($Q40*1000)</f>
+        <v>158000</v>
       </c>
       <c r="B43" t="s">
         <v>19</v>
       </c>
       <c r="C43" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D43">
-        <f t="shared" ref="D43:D48" si="4">D42+($Q42*1000)</f>
-        <v>184000</v>
+        <f>D40+($Q40*1000)</f>
+        <v>158000</v>
       </c>
       <c r="E43" t="s">
         <v>19</v>
       </c>
       <c r="F43" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="G43">
-        <f t="shared" ref="G43:G48" si="5">G42+$Q42*1000</f>
-        <v>192000</v>
+        <f>G40+Q40*1000</f>
+        <v>166000</v>
       </c>
       <c r="H43" t="s">
-        <v>60</v>
+        <v>31</v>
+      </c>
+      <c r="I43" t="s">
+        <v>43</v>
       </c>
       <c r="J43">
-        <f t="shared" ref="J43:J48" si="6">J42+$Q42*1000</f>
-        <v>192000</v>
+        <f>J42+6000</f>
+        <v>166000</v>
       </c>
       <c r="K43" t="s">
-        <v>60</v>
+        <v>19</v>
+      </c>
+      <c r="L43" t="s">
+        <v>43</v>
       </c>
       <c r="M43">
-        <f t="shared" ref="M43:M48" si="7">M42+($Q42*1000)</f>
-        <v>184000</v>
+        <f>M40+($Q40*1000)</f>
+        <v>158000</v>
       </c>
       <c r="N43" t="s">
         <v>19</v>
       </c>
       <c r="O43" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="P43">
+        <f>P40+1</f>
         <v>10</v>
       </c>
       <c r="Q43">
-        <v>35</v>
+        <v>6</v>
+      </c>
+      <c r="R43" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A44">
-        <f t="shared" si="3"/>
-        <v>219000</v>
+        <f t="shared" ref="A44:A49" si="3">A43+($Q43*1000)</f>
+        <v>164000</v>
       </c>
       <c r="B44" t="s">
         <v>19</v>
       </c>
       <c r="C44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D44">
-        <f t="shared" si="4"/>
-        <v>219000</v>
+        <f t="shared" ref="D44:D49" si="4">D43+($Q43*1000)</f>
+        <v>164000</v>
       </c>
       <c r="E44" t="s">
         <v>19</v>
       </c>
       <c r="F44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G44">
-        <f t="shared" si="5"/>
-        <v>227000</v>
+        <f t="shared" ref="G44:G49" si="5">G43+$Q43*1000</f>
+        <v>172000</v>
       </c>
       <c r="H44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J44">
-        <f t="shared" si="6"/>
-        <v>227000</v>
+        <f t="shared" ref="J44:J49" si="6">J43+$Q43*1000</f>
+        <v>172000</v>
       </c>
       <c r="K44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M44">
-        <f t="shared" si="7"/>
-        <v>219000</v>
+        <f t="shared" ref="M44:M49" si="7">M43+($Q43*1000)</f>
+        <v>164000</v>
       </c>
       <c r="N44" t="s">
         <v>19</v>
       </c>
       <c r="O44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P44">
+        <f>P43+1</f>
         <v>11</v>
       </c>
       <c r="Q44">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A45">
         <f t="shared" si="3"/>
-        <v>240000</v>
+        <v>199000</v>
       </c>
       <c r="B45" t="s">
         <v>19</v>
       </c>
       <c r="C45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D45">
         <f t="shared" si="4"/>
-        <v>240000</v>
+        <v>199000</v>
       </c>
       <c r="E45" t="s">
         <v>19</v>
       </c>
       <c r="F45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G45">
         <f t="shared" si="5"/>
-        <v>248000</v>
+        <v>207000</v>
       </c>
       <c r="H45" t="s">
         <v>62</v>
       </c>
       <c r="J45">
         <f t="shared" si="6"/>
-        <v>248000</v>
+        <v>207000</v>
       </c>
       <c r="K45" t="s">
-        <v>31</v>
-      </c>
-      <c r="L45" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="M45">
         <f t="shared" si="7"/>
-        <v>240000</v>
+        <v>199000</v>
       </c>
       <c r="N45" t="s">
         <v>19</v>
       </c>
       <c r="O45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P45">
+        <f t="shared" ref="P45:P49" si="8">P44+1</f>
         <v>12</v>
       </c>
       <c r="Q45">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A46">
         <f t="shared" si="3"/>
-        <v>244000</v>
+        <v>220000</v>
       </c>
       <c r="B46" t="s">
         <v>19</v>
@@ -2710,7 +2712,7 @@
       </c>
       <c r="D46">
         <f t="shared" si="4"/>
-        <v>244000</v>
+        <v>220000</v>
       </c>
       <c r="E46" t="s">
         <v>19</v>
@@ -2720,17 +2722,14 @@
       </c>
       <c r="G46">
         <f t="shared" si="5"/>
-        <v>252000</v>
+        <v>228000</v>
       </c>
       <c r="H46" t="s">
-        <v>31</v>
-      </c>
-      <c r="I46" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="J46">
         <f t="shared" si="6"/>
-        <v>252000</v>
+        <v>228000</v>
       </c>
       <c r="K46" t="s">
         <v>31</v>
@@ -2740,7 +2739,7 @@
       </c>
       <c r="M46">
         <f t="shared" si="7"/>
-        <v>244000</v>
+        <v>220000</v>
       </c>
       <c r="N46" t="s">
         <v>19</v>
@@ -2749,6 +2748,7 @@
         <v>48</v>
       </c>
       <c r="P46">
+        <f t="shared" si="8"/>
         <v>13</v>
       </c>
       <c r="Q46">
@@ -2758,1108 +2758,1176 @@
     <row r="47" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A47">
         <f t="shared" si="3"/>
-        <v>248000</v>
+        <v>224000</v>
       </c>
       <c r="B47" t="s">
         <v>19</v>
       </c>
       <c r="C47" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D47">
         <f t="shared" si="4"/>
-        <v>248000</v>
+        <v>224000</v>
       </c>
       <c r="E47" t="s">
         <v>19</v>
       </c>
       <c r="F47" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G47">
         <f t="shared" si="5"/>
-        <v>256000</v>
+        <v>232000</v>
       </c>
       <c r="H47" t="s">
         <v>31</v>
       </c>
       <c r="I47" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J47">
         <f t="shared" si="6"/>
-        <v>256000</v>
+        <v>232000</v>
       </c>
       <c r="K47" t="s">
         <v>31</v>
       </c>
       <c r="L47" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="M47">
         <f t="shared" si="7"/>
-        <v>248000</v>
+        <v>224000</v>
       </c>
       <c r="N47" t="s">
         <v>19</v>
       </c>
       <c r="O47" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="P47">
+        <f t="shared" si="8"/>
         <v>14</v>
       </c>
       <c r="Q47">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A48">
         <f t="shared" si="3"/>
-        <v>250000</v>
+        <v>228000</v>
       </c>
       <c r="B48" t="s">
         <v>19</v>
       </c>
       <c r="C48" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D48">
         <f t="shared" si="4"/>
-        <v>250000</v>
+        <v>228000</v>
       </c>
       <c r="E48" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F48" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G48">
         <f t="shared" si="5"/>
-        <v>258000</v>
+        <v>236000</v>
       </c>
       <c r="H48" t="s">
         <v>31</v>
       </c>
       <c r="I48" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="J48">
         <f t="shared" si="6"/>
-        <v>258000</v>
+        <v>236000</v>
       </c>
       <c r="K48" t="s">
         <v>31</v>
       </c>
       <c r="L48" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="M48">
         <f t="shared" si="7"/>
-        <v>250000</v>
+        <v>228000</v>
       </c>
       <c r="N48" t="s">
         <v>19</v>
       </c>
       <c r="O48" t="s">
+        <v>50</v>
+      </c>
+      <c r="P48">
+        <f t="shared" si="8"/>
+        <v>15</v>
+      </c>
+      <c r="Q48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <f t="shared" si="3"/>
+        <v>230000</v>
+      </c>
+      <c r="B49" t="s">
+        <v>19</v>
+      </c>
+      <c r="C49" t="s">
         <v>30</v>
       </c>
-      <c r="P48">
-        <v>15</v>
-      </c>
-      <c r="Q48">
+      <c r="D49">
+        <f t="shared" si="4"/>
+        <v>230000</v>
+      </c>
+      <c r="E49" t="s">
+        <v>31</v>
+      </c>
+      <c r="F49" t="s">
+        <v>52</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="5"/>
+        <v>238000</v>
+      </c>
+      <c r="H49" t="s">
+        <v>31</v>
+      </c>
+      <c r="I49" t="s">
+        <v>32</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="6"/>
+        <v>238000</v>
+      </c>
+      <c r="K49" t="s">
+        <v>31</v>
+      </c>
+      <c r="L49" t="s">
+        <v>33</v>
+      </c>
+      <c r="M49">
+        <f t="shared" si="7"/>
+        <v>230000</v>
+      </c>
+      <c r="N49" t="s">
+        <v>19</v>
+      </c>
+      <c r="O49" t="s">
+        <v>30</v>
+      </c>
+      <c r="P49">
+        <f t="shared" si="8"/>
+        <v>16</v>
+      </c>
+      <c r="Q49">
         <v>24</v>
-      </c>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="D49">
-        <f>D48+($S$2*(1-$R$2))</f>
-        <v>253950</v>
-      </c>
-      <c r="E49" t="s">
-        <v>19</v>
-      </c>
-      <c r="F49" t="s">
-        <v>53</v>
-      </c>
-      <c r="G49">
-        <f t="shared" ref="G49:G66" si="8">G48+($S$2)</f>
-        <v>262000</v>
-      </c>
-      <c r="H49" t="s">
-        <v>19</v>
-      </c>
-      <c r="I49" t="s">
-        <v>34</v>
-      </c>
-      <c r="J49">
-        <f>J48+($S$2*(1+$R$2))</f>
-        <v>262050</v>
-      </c>
-      <c r="K49" t="s">
-        <v>19</v>
-      </c>
-      <c r="L49" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D50">
         <f>D49+($S$2*(1-$R$2))</f>
-        <v>257900</v>
+        <v>233950</v>
       </c>
       <c r="E50" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F50" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G50">
-        <f t="shared" si="8"/>
-        <v>266000</v>
+        <f t="shared" ref="G50:G67" si="9">G49+($S$2)</f>
+        <v>242000</v>
       </c>
       <c r="H50" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I50" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J50">
-        <f t="shared" ref="J50:J69" si="9">J49+($S$2*(1+$R$2))</f>
-        <v>266100</v>
+        <f>J49+($S$2*(1+$R$2))</f>
+        <v>242050</v>
       </c>
       <c r="K50" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L50" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D51">
-        <f t="shared" ref="D51:D72" si="10">D50+($S$2*(1-$R$2))</f>
-        <v>261850</v>
+        <f>D50+($S$2*(1-$R$2))</f>
+        <v>237900</v>
       </c>
       <c r="E51" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G51">
-        <f t="shared" si="8"/>
-        <v>270000</v>
+        <f t="shared" si="9"/>
+        <v>246000</v>
       </c>
       <c r="H51" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I51" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J51">
-        <f t="shared" si="9"/>
-        <v>270150</v>
+        <f t="shared" ref="J51:J70" si="10">J50+($S$2*(1+$R$2))</f>
+        <v>246100</v>
       </c>
       <c r="K51" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L51" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D52">
+        <f t="shared" ref="D52:D73" si="11">D51+($S$2*(1-$R$2))</f>
+        <v>241850</v>
+      </c>
+      <c r="E52" t="s">
+        <v>19</v>
+      </c>
+      <c r="F52" t="s">
+        <v>53</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="9"/>
+        <v>250000</v>
+      </c>
+      <c r="H52" t="s">
+        <v>19</v>
+      </c>
+      <c r="I52" t="s">
+        <v>34</v>
+      </c>
+      <c r="J52">
         <f t="shared" si="10"/>
-        <v>265800</v>
-      </c>
-      <c r="E52" t="s">
-        <v>31</v>
-      </c>
-      <c r="F52" t="s">
-        <v>52</v>
-      </c>
-      <c r="G52">
-        <f t="shared" si="8"/>
-        <v>274000</v>
-      </c>
-      <c r="H52" t="s">
-        <v>31</v>
-      </c>
-      <c r="I52" t="s">
-        <v>32</v>
-      </c>
-      <c r="J52">
-        <f t="shared" si="9"/>
-        <v>274200</v>
+        <v>250150</v>
       </c>
       <c r="K52" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L52" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D53">
+        <f t="shared" si="11"/>
+        <v>245800</v>
+      </c>
+      <c r="E53" t="s">
+        <v>31</v>
+      </c>
+      <c r="F53" t="s">
+        <v>52</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="9"/>
+        <v>254000</v>
+      </c>
+      <c r="H53" t="s">
+        <v>31</v>
+      </c>
+      <c r="I53" t="s">
+        <v>32</v>
+      </c>
+      <c r="J53">
         <f t="shared" si="10"/>
-        <v>269750</v>
-      </c>
-      <c r="E53" t="s">
-        <v>19</v>
-      </c>
-      <c r="F53" t="s">
+        <v>254200</v>
+      </c>
+      <c r="K53" t="s">
+        <v>31</v>
+      </c>
+      <c r="L53" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="D54">
+        <f t="shared" si="11"/>
+        <v>249750</v>
+      </c>
+      <c r="E54" t="s">
+        <v>19</v>
+      </c>
+      <c r="F54" t="s">
         <v>53</v>
       </c>
-      <c r="G53">
-        <f t="shared" si="8"/>
-        <v>278000</v>
-      </c>
-      <c r="H53" t="s">
-        <v>19</v>
-      </c>
-      <c r="I53" t="s">
+      <c r="G54">
+        <f t="shared" si="9"/>
+        <v>258000</v>
+      </c>
+      <c r="H54" t="s">
+        <v>19</v>
+      </c>
+      <c r="I54" t="s">
         <v>34</v>
       </c>
-      <c r="J53">
+      <c r="J54">
+        <f t="shared" si="10"/>
+        <v>258250</v>
+      </c>
+      <c r="K54" t="s">
+        <v>19</v>
+      </c>
+      <c r="L54" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <f>A49+(Q49*1000)-((G54-D55)*0.5)</f>
+        <v>251850</v>
+      </c>
+      <c r="B55" t="s">
+        <v>31</v>
+      </c>
+      <c r="C55" t="s">
+        <v>39</v>
+      </c>
+      <c r="D55">
+        <f t="shared" si="11"/>
+        <v>253700</v>
+      </c>
+      <c r="E55" t="s">
+        <v>31</v>
+      </c>
+      <c r="F55" t="s">
+        <v>52</v>
+      </c>
+      <c r="G55">
         <f t="shared" si="9"/>
-        <v>278250</v>
-      </c>
-      <c r="K53" t="s">
-        <v>19</v>
-      </c>
-      <c r="L53" t="s">
+        <v>262000</v>
+      </c>
+      <c r="H55" t="s">
+        <v>31</v>
+      </c>
+      <c r="I55" t="s">
+        <v>32</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="10"/>
+        <v>262300</v>
+      </c>
+      <c r="K55" t="s">
+        <v>31</v>
+      </c>
+      <c r="L55" t="s">
+        <v>33</v>
+      </c>
+      <c r="M55">
+        <f>M49+($Q49*1000)</f>
+        <v>254000</v>
+      </c>
+      <c r="N55" t="s">
+        <v>19</v>
+      </c>
+      <c r="O55" t="s">
+        <v>36</v>
+      </c>
+      <c r="P55">
+        <f>P49+1</f>
+        <v>17</v>
+      </c>
+      <c r="Q55">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="D56">
+        <f t="shared" si="11"/>
+        <v>257650</v>
+      </c>
+      <c r="E56" t="s">
+        <v>19</v>
+      </c>
+      <c r="F56" t="s">
+        <v>53</v>
+      </c>
+      <c r="G56">
+        <f t="shared" si="9"/>
+        <v>266000</v>
+      </c>
+      <c r="H56" t="s">
+        <v>19</v>
+      </c>
+      <c r="I56" t="s">
+        <v>34</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="10"/>
+        <v>266350</v>
+      </c>
+      <c r="K56" t="s">
+        <v>19</v>
+      </c>
+      <c r="L56" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A54">
-        <f>A48+(Q48*1000)-((G53-D54)*0.5)</f>
-        <v>271850</v>
-      </c>
-      <c r="B54" t="s">
-        <v>31</v>
-      </c>
-      <c r="C54" t="s">
-        <v>39</v>
-      </c>
-      <c r="D54">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>66</v>
+      </c>
+      <c r="D57">
+        <f t="shared" si="11"/>
+        <v>261600</v>
+      </c>
+      <c r="E57" t="s">
+        <v>31</v>
+      </c>
+      <c r="F57" t="s">
+        <v>52</v>
+      </c>
+      <c r="G57">
+        <f t="shared" si="9"/>
+        <v>270000</v>
+      </c>
+      <c r="H57" t="s">
+        <v>31</v>
+      </c>
+      <c r="I57" t="s">
+        <v>32</v>
+      </c>
+      <c r="J57">
         <f t="shared" si="10"/>
-        <v>273700</v>
-      </c>
-      <c r="E54" t="s">
-        <v>31</v>
-      </c>
-      <c r="F54" t="s">
-        <v>52</v>
-      </c>
-      <c r="G54">
-        <f t="shared" si="8"/>
-        <v>282000</v>
-      </c>
-      <c r="H54" t="s">
-        <v>31</v>
-      </c>
-      <c r="I54" t="s">
-        <v>32</v>
-      </c>
-      <c r="J54">
-        <f t="shared" si="9"/>
-        <v>282300</v>
-      </c>
-      <c r="K54" t="s">
-        <v>31</v>
-      </c>
-      <c r="L54" t="s">
+        <v>270400</v>
+      </c>
+      <c r="K57" t="s">
+        <v>31</v>
+      </c>
+      <c r="L57" t="s">
         <v>33</v>
-      </c>
-      <c r="M54">
-        <f>M48+($Q48*1000)</f>
-        <v>274000</v>
-      </c>
-      <c r="N54" t="s">
-        <v>19</v>
-      </c>
-      <c r="O54" t="s">
-        <v>36</v>
-      </c>
-      <c r="P54">
-        <v>16</v>
-      </c>
-      <c r="Q54">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="D55">
-        <f t="shared" si="10"/>
-        <v>277650</v>
-      </c>
-      <c r="E55" t="s">
-        <v>19</v>
-      </c>
-      <c r="F55" t="s">
-        <v>53</v>
-      </c>
-      <c r="G55">
-        <f t="shared" si="8"/>
-        <v>286000</v>
-      </c>
-      <c r="H55" t="s">
-        <v>19</v>
-      </c>
-      <c r="I55" t="s">
-        <v>34</v>
-      </c>
-      <c r="J55">
-        <f t="shared" si="9"/>
-        <v>286350</v>
-      </c>
-      <c r="K55" t="s">
-        <v>19</v>
-      </c>
-      <c r="L55" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>66</v>
-      </c>
-      <c r="D56">
-        <f t="shared" si="10"/>
-        <v>281600</v>
-      </c>
-      <c r="E56" t="s">
-        <v>31</v>
-      </c>
-      <c r="F56" t="s">
-        <v>52</v>
-      </c>
-      <c r="G56">
-        <f t="shared" si="8"/>
-        <v>290000</v>
-      </c>
-      <c r="H56" t="s">
-        <v>31</v>
-      </c>
-      <c r="I56" t="s">
-        <v>32</v>
-      </c>
-      <c r="J56">
-        <f t="shared" si="9"/>
-        <v>290400</v>
-      </c>
-      <c r="K56" t="s">
-        <v>31</v>
-      </c>
-      <c r="L56" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A57">
-        <f>G48+($S$2*(1-$R$2*2))*10</f>
-        <v>297000</v>
-      </c>
-      <c r="B57" t="s">
-        <v>19</v>
-      </c>
-      <c r="C57" t="s">
-        <v>54</v>
-      </c>
-      <c r="D57">
-        <f t="shared" si="10"/>
-        <v>285550</v>
-      </c>
-      <c r="E57" t="s">
-        <v>19</v>
-      </c>
-      <c r="F57" t="s">
-        <v>53</v>
-      </c>
-      <c r="G57">
-        <f t="shared" si="8"/>
-        <v>294000</v>
-      </c>
-      <c r="H57" t="s">
-        <v>19</v>
-      </c>
-      <c r="I57" t="s">
-        <v>34</v>
-      </c>
-      <c r="J57">
-        <f t="shared" si="9"/>
-        <v>294450</v>
-      </c>
-      <c r="K57" t="s">
-        <v>19</v>
-      </c>
-      <c r="L57" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58">
-        <f t="shared" ref="A58:A71" si="11">A57+($S$2*(1-$R$2*2))</f>
-        <v>300900</v>
+        <f>G49+($S$2*(1-$R$2*2))*10</f>
+        <v>277000</v>
       </c>
       <c r="B58" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C58" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D58">
+        <f t="shared" si="11"/>
+        <v>265550</v>
+      </c>
+      <c r="E58" t="s">
+        <v>19</v>
+      </c>
+      <c r="F58" t="s">
+        <v>53</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="9"/>
+        <v>274000</v>
+      </c>
+      <c r="H58" t="s">
+        <v>19</v>
+      </c>
+      <c r="I58" t="s">
+        <v>34</v>
+      </c>
+      <c r="J58">
         <f t="shared" si="10"/>
-        <v>289500</v>
-      </c>
-      <c r="E58" t="s">
-        <v>31</v>
-      </c>
-      <c r="F58" t="s">
-        <v>52</v>
-      </c>
-      <c r="G58">
-        <f t="shared" si="8"/>
-        <v>298000</v>
-      </c>
-      <c r="H58" t="s">
-        <v>31</v>
-      </c>
-      <c r="I58" t="s">
-        <v>32</v>
-      </c>
-      <c r="J58">
-        <f t="shared" si="9"/>
-        <v>298500</v>
+        <v>274450</v>
       </c>
       <c r="K58" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L58" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59">
+        <f t="shared" ref="A59:A72" si="12">A58+($S$2*(1-$R$2*2))</f>
+        <v>280900</v>
+      </c>
+      <c r="B59" t="s">
+        <v>31</v>
+      </c>
+      <c r="C59" t="s">
+        <v>55</v>
+      </c>
+      <c r="D59">
         <f t="shared" si="11"/>
-        <v>304800</v>
-      </c>
-      <c r="B59" t="s">
-        <v>19</v>
-      </c>
-      <c r="C59" t="s">
-        <v>54</v>
-      </c>
-      <c r="D59">
+        <v>269500</v>
+      </c>
+      <c r="E59" t="s">
+        <v>31</v>
+      </c>
+      <c r="F59" t="s">
+        <v>52</v>
+      </c>
+      <c r="G59">
+        <f t="shared" si="9"/>
+        <v>278000</v>
+      </c>
+      <c r="H59" t="s">
+        <v>31</v>
+      </c>
+      <c r="I59" t="s">
+        <v>32</v>
+      </c>
+      <c r="J59">
         <f t="shared" si="10"/>
-        <v>293450</v>
-      </c>
-      <c r="E59" t="s">
-        <v>19</v>
-      </c>
-      <c r="F59" t="s">
-        <v>53</v>
-      </c>
-      <c r="G59">
-        <f t="shared" si="8"/>
-        <v>302000</v>
-      </c>
-      <c r="H59" t="s">
-        <v>19</v>
-      </c>
-      <c r="I59" t="s">
-        <v>34</v>
-      </c>
-      <c r="J59">
-        <f t="shared" si="9"/>
-        <v>302550</v>
+        <v>278500</v>
       </c>
       <c r="K59" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L59" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60">
+        <f t="shared" si="12"/>
+        <v>284800</v>
+      </c>
+      <c r="B60" t="s">
+        <v>19</v>
+      </c>
+      <c r="C60" t="s">
+        <v>54</v>
+      </c>
+      <c r="D60">
         <f t="shared" si="11"/>
-        <v>308700</v>
-      </c>
-      <c r="B60" t="s">
-        <v>31</v>
-      </c>
-      <c r="C60" t="s">
-        <v>55</v>
-      </c>
-      <c r="D60">
+        <v>273450</v>
+      </c>
+      <c r="E60" t="s">
+        <v>19</v>
+      </c>
+      <c r="F60" t="s">
+        <v>53</v>
+      </c>
+      <c r="G60">
+        <f t="shared" si="9"/>
+        <v>282000</v>
+      </c>
+      <c r="H60" t="s">
+        <v>19</v>
+      </c>
+      <c r="I60" t="s">
+        <v>34</v>
+      </c>
+      <c r="J60">
         <f t="shared" si="10"/>
-        <v>297400</v>
-      </c>
-      <c r="E60" t="s">
-        <v>31</v>
-      </c>
-      <c r="F60" t="s">
-        <v>52</v>
-      </c>
-      <c r="G60">
-        <f t="shared" si="8"/>
-        <v>306000</v>
-      </c>
-      <c r="H60" t="s">
-        <v>31</v>
-      </c>
-      <c r="I60" t="s">
-        <v>32</v>
-      </c>
-      <c r="J60">
-        <f t="shared" si="9"/>
-        <v>306600</v>
+        <v>282550</v>
       </c>
       <c r="K60" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L60" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61">
+        <f t="shared" si="12"/>
+        <v>288700</v>
+      </c>
+      <c r="B61" t="s">
+        <v>31</v>
+      </c>
+      <c r="C61" t="s">
+        <v>55</v>
+      </c>
+      <c r="D61">
         <f t="shared" si="11"/>
-        <v>312600</v>
-      </c>
-      <c r="B61" t="s">
-        <v>19</v>
-      </c>
-      <c r="C61" t="s">
-        <v>54</v>
-      </c>
-      <c r="D61">
+        <v>277400</v>
+      </c>
+      <c r="E61" t="s">
+        <v>31</v>
+      </c>
+      <c r="F61" t="s">
+        <v>52</v>
+      </c>
+      <c r="G61">
+        <f t="shared" si="9"/>
+        <v>286000</v>
+      </c>
+      <c r="H61" t="s">
+        <v>31</v>
+      </c>
+      <c r="I61" t="s">
+        <v>32</v>
+      </c>
+      <c r="J61">
         <f t="shared" si="10"/>
-        <v>301350</v>
-      </c>
-      <c r="E61" t="s">
-        <v>19</v>
-      </c>
-      <c r="F61" t="s">
-        <v>53</v>
-      </c>
-      <c r="G61">
-        <f t="shared" si="8"/>
-        <v>310000</v>
-      </c>
-      <c r="H61" t="s">
-        <v>19</v>
-      </c>
-      <c r="I61" t="s">
-        <v>34</v>
-      </c>
-      <c r="J61">
-        <f t="shared" si="9"/>
-        <v>310650</v>
+        <v>286600</v>
       </c>
       <c r="K61" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L61" t="s">
-        <v>35</v>
-      </c>
-      <c r="M61">
-        <f>M54+($Q54*1000)</f>
-        <v>302000</v>
-      </c>
-      <c r="N61" t="s">
-        <v>19</v>
-      </c>
-      <c r="O61" t="s">
-        <v>56</v>
-      </c>
-      <c r="P61">
-        <v>17</v>
-      </c>
-      <c r="Q61">
-        <v>20</v>
+        <v>33</v>
       </c>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A62">
+        <f t="shared" si="12"/>
+        <v>292600</v>
+      </c>
+      <c r="B62" t="s">
+        <v>19</v>
+      </c>
+      <c r="C62" t="s">
+        <v>54</v>
+      </c>
+      <c r="D62">
         <f t="shared" si="11"/>
-        <v>316500</v>
-      </c>
-      <c r="B62" t="s">
-        <v>31</v>
-      </c>
-      <c r="C62" t="s">
-        <v>55</v>
-      </c>
-      <c r="D62">
+        <v>281350</v>
+      </c>
+      <c r="E62" t="s">
+        <v>19</v>
+      </c>
+      <c r="F62" t="s">
+        <v>53</v>
+      </c>
+      <c r="G62">
+        <f t="shared" si="9"/>
+        <v>290000</v>
+      </c>
+      <c r="H62" t="s">
+        <v>19</v>
+      </c>
+      <c r="I62" t="s">
+        <v>34</v>
+      </c>
+      <c r="J62">
         <f t="shared" si="10"/>
-        <v>305300</v>
-      </c>
-      <c r="E62" t="s">
-        <v>31</v>
-      </c>
-      <c r="F62" t="s">
-        <v>52</v>
-      </c>
-      <c r="G62">
-        <f t="shared" si="8"/>
-        <v>314000</v>
-      </c>
-      <c r="H62" t="s">
-        <v>31</v>
-      </c>
-      <c r="I62" t="s">
-        <v>32</v>
-      </c>
-      <c r="J62">
-        <f t="shared" si="9"/>
-        <v>314700</v>
+        <v>290650</v>
       </c>
       <c r="K62" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L62" t="s">
-        <v>33</v>
+        <v>35</v>
+      </c>
+      <c r="M62">
+        <f>M55+($Q55*1000)</f>
+        <v>282000</v>
+      </c>
+      <c r="N62" t="s">
+        <v>19</v>
+      </c>
+      <c r="O62" t="s">
+        <v>56</v>
+      </c>
+      <c r="P62">
+        <f>P55+1</f>
+        <v>18</v>
+      </c>
+      <c r="Q62">
+        <v>20</v>
       </c>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A63">
+        <f t="shared" si="12"/>
+        <v>296500</v>
+      </c>
+      <c r="B63" t="s">
+        <v>31</v>
+      </c>
+      <c r="C63" t="s">
+        <v>55</v>
+      </c>
+      <c r="D63">
         <f t="shared" si="11"/>
-        <v>320400</v>
-      </c>
-      <c r="B63" t="s">
-        <v>19</v>
-      </c>
-      <c r="C63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D63">
+        <v>285300</v>
+      </c>
+      <c r="E63" t="s">
+        <v>31</v>
+      </c>
+      <c r="F63" t="s">
+        <v>52</v>
+      </c>
+      <c r="G63">
+        <f t="shared" si="9"/>
+        <v>294000</v>
+      </c>
+      <c r="H63" t="s">
+        <v>31</v>
+      </c>
+      <c r="I63" t="s">
+        <v>32</v>
+      </c>
+      <c r="J63">
         <f t="shared" si="10"/>
-        <v>309250</v>
-      </c>
-      <c r="E63" t="s">
-        <v>19</v>
-      </c>
-      <c r="F63" t="s">
-        <v>53</v>
-      </c>
-      <c r="G63">
-        <f t="shared" si="8"/>
-        <v>318000</v>
-      </c>
-      <c r="H63" t="s">
-        <v>19</v>
-      </c>
-      <c r="I63" t="s">
-        <v>34</v>
-      </c>
-      <c r="J63">
-        <f t="shared" si="9"/>
-        <v>318750</v>
+        <v>294700</v>
       </c>
       <c r="K63" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L63" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A64">
+        <f t="shared" si="12"/>
+        <v>300400</v>
+      </c>
+      <c r="B64" t="s">
+        <v>19</v>
+      </c>
+      <c r="C64" t="s">
+        <v>54</v>
+      </c>
+      <c r="D64">
         <f t="shared" si="11"/>
-        <v>324300</v>
-      </c>
-      <c r="B64" t="s">
-        <v>31</v>
-      </c>
-      <c r="C64" t="s">
-        <v>55</v>
-      </c>
-      <c r="D64">
+        <v>289250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>19</v>
+      </c>
+      <c r="F64" t="s">
+        <v>53</v>
+      </c>
+      <c r="G64">
+        <f t="shared" si="9"/>
+        <v>298000</v>
+      </c>
+      <c r="H64" t="s">
+        <v>19</v>
+      </c>
+      <c r="I64" t="s">
+        <v>34</v>
+      </c>
+      <c r="J64">
         <f t="shared" si="10"/>
-        <v>313200</v>
-      </c>
-      <c r="E64" t="s">
-        <v>31</v>
-      </c>
-      <c r="F64" t="s">
-        <v>52</v>
-      </c>
-      <c r="G64">
-        <f t="shared" si="8"/>
-        <v>322000</v>
-      </c>
-      <c r="H64" t="s">
-        <v>31</v>
-      </c>
-      <c r="I64" t="s">
-        <v>57</v>
-      </c>
-      <c r="J64">
-        <f t="shared" si="9"/>
-        <v>322800</v>
+        <v>298750</v>
       </c>
       <c r="K64" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L64" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65">
+        <f t="shared" si="12"/>
+        <v>304300</v>
+      </c>
+      <c r="B65" t="s">
+        <v>31</v>
+      </c>
+      <c r="C65" t="s">
+        <v>55</v>
+      </c>
+      <c r="D65">
         <f t="shared" si="11"/>
-        <v>328200</v>
-      </c>
-      <c r="B65" t="s">
-        <v>19</v>
-      </c>
-      <c r="C65" t="s">
-        <v>54</v>
-      </c>
-      <c r="D65">
+        <v>293200</v>
+      </c>
+      <c r="E65" t="s">
+        <v>31</v>
+      </c>
+      <c r="F65" t="s">
+        <v>52</v>
+      </c>
+      <c r="G65">
+        <f t="shared" si="9"/>
+        <v>302000</v>
+      </c>
+      <c r="H65" t="s">
+        <v>31</v>
+      </c>
+      <c r="I65" t="s">
+        <v>57</v>
+      </c>
+      <c r="J65">
         <f t="shared" si="10"/>
-        <v>317150</v>
-      </c>
-      <c r="E65" t="s">
-        <v>19</v>
-      </c>
-      <c r="F65" t="s">
-        <v>53</v>
-      </c>
-      <c r="G65">
-        <f t="shared" si="8"/>
-        <v>326000</v>
-      </c>
-      <c r="H65" t="s">
-        <v>19</v>
-      </c>
-      <c r="I65" t="s">
-        <v>43</v>
-      </c>
-      <c r="J65">
-        <f t="shared" si="9"/>
-        <v>326850</v>
+        <v>302800</v>
       </c>
       <c r="K65" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L65" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66">
+        <f t="shared" si="12"/>
+        <v>308200</v>
+      </c>
+      <c r="B66" t="s">
+        <v>19</v>
+      </c>
+      <c r="C66" t="s">
+        <v>54</v>
+      </c>
+      <c r="D66">
         <f t="shared" si="11"/>
-        <v>332100</v>
-      </c>
-      <c r="B66" t="s">
-        <v>31</v>
-      </c>
-      <c r="C66" t="s">
-        <v>55</v>
-      </c>
-      <c r="D66">
+        <v>297150</v>
+      </c>
+      <c r="E66" t="s">
+        <v>19</v>
+      </c>
+      <c r="F66" t="s">
+        <v>53</v>
+      </c>
+      <c r="G66">
+        <f t="shared" si="9"/>
+        <v>306000</v>
+      </c>
+      <c r="H66" t="s">
+        <v>19</v>
+      </c>
+      <c r="I66" t="s">
+        <v>43</v>
+      </c>
+      <c r="J66">
         <f t="shared" si="10"/>
-        <v>321100</v>
-      </c>
-      <c r="E66" t="s">
-        <v>31</v>
-      </c>
-      <c r="F66" t="s">
-        <v>52</v>
-      </c>
-      <c r="G66">
-        <f t="shared" si="8"/>
-        <v>330000</v>
-      </c>
-      <c r="H66" t="s">
-        <v>60</v>
-      </c>
-      <c r="J66">
-        <f t="shared" si="9"/>
-        <v>330900</v>
+        <v>306850</v>
       </c>
       <c r="K66" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L66" t="s">
-        <v>33</v>
-      </c>
-      <c r="M66">
-        <f>M61+($Q61*1000)</f>
-        <v>322000</v>
-      </c>
-      <c r="N66" t="s">
-        <v>19</v>
-      </c>
-      <c r="O66" t="s">
-        <v>41</v>
-      </c>
-      <c r="P66">
-        <v>18</v>
-      </c>
-      <c r="Q66">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A67">
+        <f t="shared" si="12"/>
+        <v>312100</v>
+      </c>
+      <c r="B67" t="s">
+        <v>31</v>
+      </c>
+      <c r="C67" t="s">
+        <v>55</v>
+      </c>
+      <c r="D67">
         <f t="shared" si="11"/>
-        <v>336000</v>
-      </c>
-      <c r="B67" t="s">
-        <v>19</v>
-      </c>
-      <c r="C67" t="s">
-        <v>54</v>
-      </c>
-      <c r="D67">
+        <v>301100</v>
+      </c>
+      <c r="E67" t="s">
+        <v>31</v>
+      </c>
+      <c r="F67" t="s">
+        <v>52</v>
+      </c>
+      <c r="G67">
+        <f t="shared" si="9"/>
+        <v>310000</v>
+      </c>
+      <c r="H67" t="s">
+        <v>60</v>
+      </c>
+      <c r="J67">
         <f t="shared" si="10"/>
-        <v>325050</v>
-      </c>
-      <c r="E67" t="s">
-        <v>19</v>
-      </c>
-      <c r="F67" t="s">
-        <v>53</v>
-      </c>
-      <c r="J67">
-        <f t="shared" si="9"/>
-        <v>334950</v>
+        <v>310900</v>
       </c>
       <c r="K67" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L67" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="M67">
+        <f>M62+($Q62*1000)</f>
+        <v>302000</v>
+      </c>
+      <c r="N67" t="s">
+        <v>19</v>
+      </c>
+      <c r="O67" t="s">
+        <v>41</v>
+      </c>
+      <c r="P67">
+        <f>P62+1</f>
+        <v>19</v>
+      </c>
+      <c r="Q67">
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A68">
+        <f t="shared" si="12"/>
+        <v>316000</v>
+      </c>
+      <c r="B68" t="s">
+        <v>19</v>
+      </c>
+      <c r="C68" t="s">
+        <v>54</v>
+      </c>
+      <c r="D68">
         <f t="shared" si="11"/>
-        <v>339900</v>
-      </c>
-      <c r="B68" t="s">
-        <v>31</v>
-      </c>
-      <c r="C68" t="s">
-        <v>55</v>
-      </c>
-      <c r="D68">
+        <v>305050</v>
+      </c>
+      <c r="E68" t="s">
+        <v>19</v>
+      </c>
+      <c r="F68" t="s">
+        <v>53</v>
+      </c>
+      <c r="J68">
         <f t="shared" si="10"/>
-        <v>329000</v>
-      </c>
-      <c r="E68" t="s">
-        <v>31</v>
-      </c>
-      <c r="F68" t="s">
-        <v>52</v>
-      </c>
-      <c r="G68">
-        <f>G66+$Q66*1000</f>
-        <v>340000</v>
-      </c>
-      <c r="H68" t="s">
-        <v>60</v>
-      </c>
-      <c r="J68">
-        <f t="shared" si="9"/>
-        <v>339000</v>
+        <v>314950</v>
       </c>
       <c r="K68" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L68" t="s">
-        <v>33</v>
-      </c>
-      <c r="M68">
-        <f>M66+($Q66*1000)</f>
-        <v>332000</v>
-      </c>
-      <c r="N68" t="s">
-        <v>19</v>
-      </c>
-      <c r="O68" t="s">
-        <v>58</v>
-      </c>
-      <c r="P68">
-        <v>19</v>
-      </c>
-      <c r="Q68">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A69">
+        <f t="shared" si="12"/>
+        <v>319900</v>
+      </c>
+      <c r="B69" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" t="s">
+        <v>55</v>
+      </c>
+      <c r="D69">
         <f t="shared" si="11"/>
-        <v>343800</v>
-      </c>
-      <c r="B69" t="s">
-        <v>19</v>
-      </c>
-      <c r="C69" t="s">
-        <v>54</v>
-      </c>
-      <c r="D69">
+        <v>309000</v>
+      </c>
+      <c r="E69" t="s">
+        <v>31</v>
+      </c>
+      <c r="F69" t="s">
+        <v>52</v>
+      </c>
+      <c r="G69">
+        <f>G67+$Q67*1000</f>
+        <v>320000</v>
+      </c>
+      <c r="H69" t="s">
+        <v>60</v>
+      </c>
+      <c r="J69">
         <f t="shared" si="10"/>
-        <v>332950</v>
-      </c>
-      <c r="E69" t="s">
-        <v>19</v>
-      </c>
-      <c r="F69" t="s">
-        <v>53</v>
-      </c>
-      <c r="J69">
-        <f t="shared" si="9"/>
-        <v>343050</v>
+        <v>319000</v>
       </c>
       <c r="K69" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L69" t="s">
-        <v>43</v>
+        <v>33</v>
+      </c>
+      <c r="M69">
+        <f>M67+($Q67*1000)</f>
+        <v>312000</v>
+      </c>
+      <c r="N69" t="s">
+        <v>19</v>
+      </c>
+      <c r="O69" t="s">
+        <v>58</v>
+      </c>
+      <c r="P69">
+        <f>P67+1</f>
+        <v>20</v>
+      </c>
+      <c r="Q69">
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A70">
+        <f t="shared" si="12"/>
+        <v>323800</v>
+      </c>
+      <c r="B70" t="s">
+        <v>19</v>
+      </c>
+      <c r="C70" t="s">
+        <v>54</v>
+      </c>
+      <c r="D70">
         <f t="shared" si="11"/>
-        <v>347700</v>
-      </c>
-      <c r="B70" t="s">
-        <v>31</v>
-      </c>
-      <c r="C70" t="s">
-        <v>59</v>
-      </c>
-      <c r="D70">
+        <v>312950</v>
+      </c>
+      <c r="E70" t="s">
+        <v>19</v>
+      </c>
+      <c r="F70" t="s">
+        <v>53</v>
+      </c>
+      <c r="J70">
         <f t="shared" si="10"/>
-        <v>336900</v>
-      </c>
-      <c r="E70" t="s">
-        <v>31</v>
-      </c>
-      <c r="F70" t="s">
-        <v>52</v>
-      </c>
-      <c r="J70">
-        <f>J69+($S$2*(1+$R$2))</f>
-        <v>347100</v>
+        <v>323050</v>
       </c>
       <c r="K70" t="s">
-        <v>60</v>
+        <v>19</v>
+      </c>
+      <c r="L70" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A71">
+        <f t="shared" si="12"/>
+        <v>327700</v>
+      </c>
+      <c r="B71" t="s">
+        <v>31</v>
+      </c>
+      <c r="C71" t="s">
+        <v>59</v>
+      </c>
+      <c r="D71">
         <f t="shared" si="11"/>
-        <v>351600</v>
-      </c>
-      <c r="B71" t="s">
+        <v>316900</v>
+      </c>
+      <c r="E71" t="s">
+        <v>31</v>
+      </c>
+      <c r="F71" t="s">
+        <v>52</v>
+      </c>
+      <c r="J71">
+        <f>J70+($S$2*(1+$R$2))</f>
+        <v>327100</v>
+      </c>
+      <c r="K71" t="s">
         <v>60</v>
       </c>
-      <c r="D71">
-        <f t="shared" si="10"/>
-        <v>340850</v>
-      </c>
-      <c r="E71" t="s">
-        <v>19</v>
-      </c>
-      <c r="F71" t="s">
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <f t="shared" si="12"/>
+        <v>331600</v>
+      </c>
+      <c r="B72" t="s">
+        <v>60</v>
+      </c>
+      <c r="D72">
+        <f t="shared" si="11"/>
+        <v>320850</v>
+      </c>
+      <c r="E72" t="s">
+        <v>19</v>
+      </c>
+      <c r="F72" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="D72">
-        <f t="shared" si="10"/>
-        <v>344800</v>
-      </c>
-      <c r="E72" t="s">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="D73">
+        <f t="shared" si="11"/>
+        <v>324800</v>
+      </c>
+      <c r="E73" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="G73">
-        <f>G68+$Q68*1000</f>
-        <v>355000</v>
-      </c>
-      <c r="H73" t="s">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="G74">
+        <f>G69+$Q69*1000</f>
+        <v>335000</v>
+      </c>
+      <c r="H74" t="s">
         <v>62</v>
       </c>
-      <c r="M73">
-        <f>M68+($Q68*1000)</f>
-        <v>347000</v>
-      </c>
-      <c r="N73" t="s">
-        <v>19</v>
-      </c>
-      <c r="O73" t="s">
+      <c r="M74">
+        <f>M69+($Q69*1000)</f>
+        <v>327000</v>
+      </c>
+      <c r="N74" t="s">
+        <v>19</v>
+      </c>
+      <c r="O74" t="s">
         <v>61</v>
       </c>
-      <c r="P73">
-        <v>20</v>
-      </c>
-      <c r="Q73">
+      <c r="P74">
+        <f>P69+1</f>
+        <v>21</v>
+      </c>
+      <c r="Q74">
         <v>40</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="J82">
-        <f>J70+Q73*1000</f>
-        <v>387100</v>
-      </c>
-      <c r="K82" t="s">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="J83">
+        <f>J71+Q74*1000</f>
+        <v>367100</v>
+      </c>
+      <c r="K83" t="s">
         <v>62</v>
       </c>
-      <c r="M82">
-        <f>M73+($Q73*1000)</f>
-        <v>387000</v>
-      </c>
-      <c r="N82" t="s">
-        <v>19</v>
-      </c>
-      <c r="O82" t="s">
+      <c r="M83">
+        <f>M74+($Q74*1000)</f>
+        <v>367000</v>
+      </c>
+      <c r="N83" t="s">
+        <v>19</v>
+      </c>
+      <c r="O83" t="s">
         <v>43</v>
       </c>
-      <c r="P82">
-        <v>21</v>
-      </c>
-      <c r="Q82">
+      <c r="P83">
+        <f>P74+1</f>
+        <v>22</v>
+      </c>
+      <c r="Q83">
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="D83">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="D84">
         <v>318500</v>
       </c>
-      <c r="E83" t="s">
+      <c r="E84" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A84">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A85">
         <v>321000</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B85" t="s">
         <v>62</v>
       </c>
-      <c r="M84">
-        <f>M82+($Q82*1000)</f>
-        <v>392000</v>
-      </c>
-      <c r="N84" t="s">
-        <v>19</v>
-      </c>
-      <c r="O84" t="s">
+      <c r="M85">
+        <f>M83+($Q83*1000)</f>
+        <v>372000</v>
+      </c>
+      <c r="N85" t="s">
+        <v>19</v>
+      </c>
+      <c r="O85" t="s">
         <v>63</v>
       </c>
-      <c r="P84">
-        <v>22</v>
-      </c>
-      <c r="Q84">
+      <c r="P85">
+        <f>P83+1</f>
+        <v>23</v>
+      </c>
+      <c r="Q85">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
onsets phone down at tacet update
</commit_message>
<xml_diff>
--- a/onsets_edit.xlsx
+++ b/onsets_edit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brandonwoosnyder/Dropbox/docs-d/00_UCI_2025-2026/02_UCI_Winter_2026/Independent Study Rajna - Music 299/Constrained_PhoneGuide_Score/ScreenTimeScore/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB062B13-947F-3A4B-B920-48B0AD36A76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07FF8F69-5DAB-8B42-A3E5-F031907A74A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{656903FE-55D6-334E-8317-D02588440573}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="85">
   <si>
     <t>onset_ms_1</t>
   </si>
@@ -287,6 +287,10 @@
   </si>
   <si>
     <t>Phone Up (3")</t>
+  </si>
+  <si>
+    <t>Phone Down
+Tacet 6"</t>
   </si>
 </sst>
 </file>
@@ -1828,7 +1832,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A14">
         <f>A13+($Q13*1000)</f>
         <v>50000</v>
@@ -1836,8 +1840,8 @@
       <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" t="s">
-        <v>59</v>
+      <c r="C14" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="D14">
         <f>D13+($Q13*1000)</f>
@@ -1846,8 +1850,8 @@
       <c r="E14" t="s">
         <v>19</v>
       </c>
-      <c r="F14" t="s">
-        <v>59</v>
+      <c r="F14" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="G14">
         <f>G13+($Q13*1000)</f>
@@ -1856,8 +1860,8 @@
       <c r="H14" t="s">
         <v>19</v>
       </c>
-      <c r="I14" t="s">
-        <v>59</v>
+      <c r="I14" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="J14">
         <f>J13+($Q13*1000)</f>
@@ -1866,8 +1870,8 @@
       <c r="K14" t="s">
         <v>19</v>
       </c>
-      <c r="L14" t="s">
-        <v>59</v>
+      <c r="L14" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="M14">
         <f>M13+($Q13*1000)</f>
@@ -1876,8 +1880,8 @@
       <c r="N14" t="s">
         <v>19</v>
       </c>
-      <c r="O14" t="s">
-        <v>59</v>
+      <c r="O14" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="P14">
         <f>P13+1</f>
@@ -4227,7 +4231,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:XFD28 J29:L31 A29:I33 M29:XFD33 K32:L33 A34:XFD1048576">
+  <conditionalFormatting sqref="J29:L31 A29:I33 M29:XFD33 K32:L33 A34:XFD1048576 A1:XFD28">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="bacon">
       <formula>NOT(ISERROR(SEARCH("bacon",A1)))</formula>
     </cfRule>

</xml_diff>